<commit_message>
banco de dados no ssms
</commit_message>
<xml_diff>
--- a/Iniciando Tabelas.xlsx
+++ b/Iniciando Tabelas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\54781547842\Desktop\Banco_de_Dados_M\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D63883F0-4365-4BF4-95EE-F93993BE3550}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2CDFBB-71B1-49CF-BC5B-CBBE187E6250}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{10CFB757-2851-4879-BCF0-C5F6210E1554}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{10CFB757-2851-4879-BCF0-C5F6210E1554}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Nome</t>
   </si>
@@ -76,12 +76,6 @@
     <t>Ezequiel</t>
   </si>
   <si>
-    <t>SaoPaulo</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
     <t>Cleide</t>
   </si>
   <si>
@@ -106,17 +100,29 @@
     <t>Ingles</t>
   </si>
   <si>
-    <t>ID Disciplinas</t>
-  </si>
-  <si>
-    <t>1,2,3</t>
+    <t>ALUNO/DISCIPLINA</t>
+  </si>
+  <si>
+    <t>ID_Aluno</t>
+  </si>
+  <si>
+    <t>ID_Disciplina</t>
+  </si>
+  <si>
+    <t>CidadeEstado</t>
+  </si>
+  <si>
+    <t>São Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,6 +174,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -195,7 +225,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -270,112 +300,298 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -387,55 +603,137 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -750,141 +1048,245 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E46BEF85-946C-45F7-8932-18E4B2E69FCA}">
-  <dimension ref="I4:R17"/>
+  <dimension ref="I4:U22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="14" max="14" width="12.33203125" customWidth="1"/>
     <col min="18" max="18" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="9:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="9:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I5" s="13" t="s">
+    <row r="4" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I5" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="47"/>
+      <c r="O5" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="23"/>
+      <c r="T5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="15"/>
-      <c r="Q5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="9:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J6" s="8" t="s">
+      <c r="U5" s="9"/>
+    </row>
+    <row r="6" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I6" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="L6" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="M6" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="N6" s="9" t="s">
+      <c r="O6" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="R6" s="19" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="9:18" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q6" s="28"/>
+      <c r="T6" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="U6" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="9:21" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I7" s="20">
         <v>1</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="49">
         <v>111</v>
       </c>
-      <c r="L7" s="18" t="s">
+      <c r="L7" s="43">
+        <v>1</v>
+      </c>
+      <c r="O7" s="20">
+        <v>1</v>
+      </c>
+      <c r="P7" s="24">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="25"/>
+      <c r="T7" s="14">
+        <v>1</v>
+      </c>
+      <c r="U7" s="51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="9:21" x14ac:dyDescent="0.3">
+      <c r="I8" s="13">
+        <v>2</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="18" t="s">
+      <c r="K8" s="7">
+        <v>222</v>
+      </c>
+      <c r="L8" s="44">
+        <v>1</v>
+      </c>
+      <c r="O8" s="13">
+        <v>1</v>
+      </c>
+      <c r="P8" s="17">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="18"/>
+      <c r="T8" s="15">
+        <v>2</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I9" s="1"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="3"/>
+      <c r="O9" s="13">
+        <v>1</v>
+      </c>
+      <c r="P9" s="17">
+        <v>3</v>
+      </c>
+      <c r="Q9" s="18"/>
+      <c r="T9" s="16">
+        <v>3</v>
+      </c>
+      <c r="U9" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I10" s="1"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="3"/>
+      <c r="O10" s="31">
+        <v>2</v>
+      </c>
+      <c r="P10" s="32">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="33"/>
+    </row>
+    <row r="11" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I11" s="4"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="6"/>
+      <c r="O11" s="34">
+        <v>2</v>
+      </c>
+      <c r="P11" s="35">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="36"/>
+    </row>
+    <row r="15" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="9:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I16" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="29"/>
+      <c r="K16" s="30"/>
+    </row>
+    <row r="17" spans="9:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I17" s="41" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="K17" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="N17" s="30"/>
+      <c r="O17" s="8"/>
+    </row>
+    <row r="18" spans="9:15" x14ac:dyDescent="0.3">
+      <c r="I18" s="37">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K18" s="43">
+        <v>1</v>
+      </c>
+      <c r="M18" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="N18" s="40" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="9:15" x14ac:dyDescent="0.3">
+      <c r="I19" s="38">
+        <v>2</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="N7" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="22">
+      <c r="K19" s="44">
         <v>1</v>
       </c>
-      <c r="R7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="9:18" x14ac:dyDescent="0.3">
-      <c r="I8" s="10">
-        <v>2</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="K8" s="11">
-        <v>222</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="N8" s="12"/>
-      <c r="Q8" s="22">
-        <v>2</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="9:18" x14ac:dyDescent="0.3">
-      <c r="I9" s="2"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="4"/>
-      <c r="Q9" s="22">
-        <v>3</v>
-      </c>
-      <c r="R9" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="9:18" x14ac:dyDescent="0.3">
-      <c r="I10" s="2"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="4"/>
-    </row>
-    <row r="11" spans="9:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I11" s="5"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="7"/>
-    </row>
-    <row r="17" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O17" s="23"/>
+      <c r="M19" s="42">
+        <v>1</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="9:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I20" s="1"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="3"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="6"/>
+    </row>
+    <row r="21" spans="9:15" x14ac:dyDescent="0.3">
+      <c r="I21" s="1"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="9:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I22" s="4"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="I5:N5"/>
+  <mergeCells count="11">
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="I5:L5"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>